<commit_message>
Revising upload teamplate for store emp
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/STORE-EMP-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/STORE-EMP-UPLOAD-TEMPLATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\node proj\rest-api-nestjs\uploads\UPLOAD-TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7DDE92-7B20-4FB6-A1D6-3D8FBCEA582B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C979D49E-58A6-474C-861A-CCEF72F7137B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15960" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>STORE IFS</t>
   </si>
@@ -85,6 +85,12 @@
   </si>
   <si>
     <t>ASSIGNMENT MONTH</t>
+  </si>
+  <si>
+    <t>ASSIGNED AC EMP. NO.</t>
+  </si>
+  <si>
+    <t>ASSIGNED AC NAME</t>
   </si>
 </sst>
 </file>
@@ -451,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE589B1-C7BA-44D4-9E29-919A5892AA9B}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -459,65 +465,73 @@
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.5703125" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>50000917</v>
       </c>
@@ -528,27 +542,33 @@
         <v>14</v>
       </c>
       <c r="D2">
+        <v>1234567</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2">
         <v>101234</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="F2">
+      <c r="H2">
         <v>102330</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="J2">
+      <c r="L2">
         <v>123456</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="2">
+      <c r="P2" s="2">
         <v>46143</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>